<commit_message>
Actualizacion automatica 2026-09-16 22:57 UTC
</commit_message>
<xml_diff>
--- a/data/50001563 - ZITRON COLOMBIA ANTIOQUIA.xlsx
+++ b/data/50001563 - ZITRON COLOMBIA ANTIOQUIA.xlsx
@@ -1627,13 +1627,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46188.509159629626</v>
+        <v>46188.634159629626</v>
       </c>
       <c r="C4" s="5">
-        <v>46188.79468755787</v>
+        <v>46188.91968755787</v>
       </c>
       <c r="D4" s="5">
-        <v>46258.03854357639</v>
+        <v>46258.16354357639</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1680,13 +1680,13 @@
         <v>28</v>
       </c>
       <c r="B5" s="9">
-        <v>46188.509310856476</v>
+        <v>46188.634310856476</v>
       </c>
       <c r="C5" s="9">
-        <v>46188.794674178236</v>
+        <v>46188.919674178236</v>
       </c>
       <c r="D5" s="9">
-        <v>46222.51097420139</v>
+        <v>46222.63597420139</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>29</v>
@@ -1745,13 +1745,13 @@
         <v>33</v>
       </c>
       <c r="B6" s="5">
-        <v>46188.50931648148</v>
+        <v>46188.63431648148</v>
       </c>
       <c r="C6" s="5">
-        <v>46188.794543298616</v>
+        <v>46188.919543298616</v>
       </c>
       <c r="D6" s="5">
-        <v>46222.510976273144</v>
+        <v>46222.635976273144</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>34</v>
@@ -1810,13 +1810,13 @@
         <v>36</v>
       </c>
       <c r="B7" s="9">
-        <v>46188.50932182871</v>
+        <v>46188.63432182871</v>
       </c>
       <c r="C7" s="9">
-        <v>46188.79459428241</v>
+        <v>46188.91959428241</v>
       </c>
       <c r="D7" s="9">
-        <v>46188.7946094213</v>
+        <v>46188.9196094213</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>37</v>
@@ -1875,13 +1875,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46188.509326643514</v>
+        <v>46188.634326643514</v>
       </c>
       <c r="C8" s="5">
-        <v>46188.794635115744</v>
+        <v>46188.919635115744</v>
       </c>
       <c r="D8" s="5">
-        <v>46188.79465210648</v>
+        <v>46188.91965210648</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1940,13 +1940,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="9">
-        <v>46188.509165474534</v>
+        <v>46188.634165474534</v>
       </c>
       <c r="C9" s="9">
-        <v>46188.79557981482</v>
+        <v>46188.92057981482</v>
       </c>
       <c r="D9" s="9">
-        <v>46188.79559026621</v>
+        <v>46188.92059026621</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>44</v>
@@ -1993,13 +1993,13 @@
         <v>46</v>
       </c>
       <c r="B10" s="5">
-        <v>46188.50933173611</v>
+        <v>46188.63433173611</v>
       </c>
       <c r="C10" s="5">
-        <v>46188.795111388885</v>
+        <v>46188.920111388885</v>
       </c>
       <c r="D10" s="5">
-        <v>46188.795113182874</v>
+        <v>46188.920113182874</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>47</v>
@@ -2058,13 +2058,13 @@
         <v>50</v>
       </c>
       <c r="B11" s="9">
-        <v>46188.50934310185</v>
+        <v>46188.63434310185</v>
       </c>
       <c r="C11" s="9">
-        <v>46188.79474537037</v>
+        <v>46188.91974537037</v>
       </c>
       <c r="D11" s="9">
-        <v>46188.79532122685</v>
+        <v>46188.92032122685</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>51</v>
@@ -2123,13 +2123,13 @@
         <v>54</v>
       </c>
       <c r="B12" s="5">
-        <v>46188.50935032408</v>
+        <v>46188.63435032408</v>
       </c>
       <c r="C12" s="5">
-        <v>46188.79548497685</v>
+        <v>46188.92048497685</v>
       </c>
       <c r="D12" s="5">
-        <v>46188.79550125</v>
+        <v>46188.92050125</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>55</v>
@@ -2188,13 +2188,13 @@
         <v>57</v>
       </c>
       <c r="B13" s="9">
-        <v>46188.509356759256</v>
+        <v>46188.634356759256</v>
       </c>
       <c r="C13" s="9">
-        <v>46188.795564201384</v>
+        <v>46188.920564201384</v>
       </c>
       <c r="D13" s="9">
-        <v>46188.79557991898</v>
+        <v>46188.92057991898</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>58</v>
@@ -2253,13 +2253,13 @@
         <v>61</v>
       </c>
       <c r="B14" s="5">
-        <v>46188.509170000005</v>
+        <v>46188.634170000005</v>
       </c>
       <c r="C14" s="5">
-        <v>46206.37878961806</v>
+        <v>46206.50378961806</v>
       </c>
       <c r="D14" s="5">
-        <v>46206.37880298611</v>
+        <v>46206.50380298611</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>62</v>
@@ -2306,13 +2306,13 @@
         <v>64</v>
       </c>
       <c r="B15" s="9">
-        <v>46188.50936615741</v>
+        <v>46188.63436615741</v>
       </c>
       <c r="C15" s="9">
-        <v>46188.79565792824</v>
+        <v>46188.92065792824</v>
       </c>
       <c r="D15" s="9">
-        <v>46189.689397685186</v>
+        <v>46189.814397685186</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>65</v>
@@ -2371,13 +2371,13 @@
         <v>67</v>
       </c>
       <c r="B16" s="5">
-        <v>46188.50937259259</v>
+        <v>46188.63437259259</v>
       </c>
       <c r="C16" s="5">
-        <v>46188.7963359375</v>
+        <v>46188.9213359375</v>
       </c>
       <c r="D16" s="5">
-        <v>46189.689421944444</v>
+        <v>46189.814421944444</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>68</v>
@@ -2436,13 +2436,13 @@
         <v>71</v>
       </c>
       <c r="B17" s="9">
-        <v>46188.50937929398</v>
+        <v>46188.63437929398</v>
       </c>
       <c r="C17" s="9">
-        <v>46197.46146039352</v>
+        <v>46197.58646039352</v>
       </c>
       <c r="D17" s="9">
-        <v>46223.43856081019</v>
+        <v>46223.56356081019</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>72</v>
@@ -2501,13 +2501,13 @@
         <v>76</v>
       </c>
       <c r="B18" s="5">
-        <v>46188.50938636574</v>
+        <v>46188.63438636574</v>
       </c>
       <c r="C18" s="5">
-        <v>46206.377370312504</v>
+        <v>46206.502370312504</v>
       </c>
       <c r="D18" s="5">
-        <v>46223.43855663194</v>
+        <v>46223.56355663194</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -2566,13 +2566,13 @@
         <v>80</v>
       </c>
       <c r="B19" s="9">
-        <v>46188.509392708336</v>
+        <v>46188.634392708336</v>
       </c>
       <c r="C19" s="9">
-        <v>46206.37854868056</v>
+        <v>46206.50354868056</v>
       </c>
       <c r="D19" s="9">
-        <v>46223.43855248843</v>
+        <v>46223.56355248843</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>81</v>
@@ -2631,13 +2631,13 @@
         <v>83</v>
       </c>
       <c r="B20" s="5">
-        <v>46188.50939828704</v>
+        <v>46188.63439828704</v>
       </c>
       <c r="C20" s="5">
-        <v>46206.37823137731</v>
+        <v>46206.50323137731</v>
       </c>
       <c r="D20" s="5">
-        <v>46223.43854857639</v>
+        <v>46223.56354857639</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>84</v>
@@ -2696,13 +2696,13 @@
         <v>86</v>
       </c>
       <c r="B21" s="9">
-        <v>46188.509403055556</v>
+        <v>46188.634403055556</v>
       </c>
       <c r="C21" s="9">
-        <v>46206.3787743287</v>
+        <v>46206.5037743287</v>
       </c>
       <c r="D21" s="9">
-        <v>46223.4385421412</v>
+        <v>46223.5635421412</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>87</v>
@@ -2761,13 +2761,13 @@
         <v>89</v>
       </c>
       <c r="B22" s="5">
-        <v>46189.65575929398</v>
+        <v>46189.78075929398</v>
       </c>
       <c r="C22" s="5">
-        <v>46197.46162379629</v>
+        <v>46197.58662379629</v>
       </c>
       <c r="D22" s="5">
-        <v>46262.8205846412</v>
+        <v>46262.9455846412</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>90</v>
@@ -2816,13 +2816,13 @@
         <v>93</v>
       </c>
       <c r="B23" s="9">
-        <v>46189.68687604167</v>
+        <v>46189.81187604167</v>
       </c>
       <c r="C23" s="9">
-        <v>46197.461606770834</v>
+        <v>46197.586606770834</v>
       </c>
       <c r="D23" s="9">
-        <v>46223.438613356484</v>
+        <v>46223.563613356484</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>94</v>
@@ -2881,13 +2881,13 @@
         <v>96</v>
       </c>
       <c r="B24" s="5">
-        <v>46189.6870440162</v>
+        <v>46189.8120440162</v>
       </c>
       <c r="C24" s="5">
-        <v>46197.46154909722</v>
+        <v>46197.58654909722</v>
       </c>
       <c r="D24" s="5">
-        <v>46223.438609467594</v>
+        <v>46223.563609467594</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>97</v>
@@ -2946,13 +2946,13 @@
         <v>99</v>
       </c>
       <c r="B25" s="9">
-        <v>46188.509174861116</v>
+        <v>46188.634174861116</v>
       </c>
       <c r="C25" s="9">
-        <v>46212.72834166666</v>
+        <v>46212.85334166666</v>
       </c>
       <c r="D25" s="9">
-        <v>46212.72836304398</v>
+        <v>46212.85336304398</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>100</v>
@@ -2999,13 +2999,13 @@
         <v>102</v>
       </c>
       <c r="B26" s="5">
-        <v>46188.50942598379</v>
+        <v>46188.63442598379</v>
       </c>
       <c r="C26" s="5">
-        <v>46212.528515659724</v>
+        <v>46212.653515659724</v>
       </c>
       <c r="D26" s="5">
-        <v>46212.528841203704</v>
+        <v>46212.653841203704</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>103</v>
@@ -3064,13 +3064,13 @@
         <v>107</v>
       </c>
       <c r="B27" s="9">
-        <v>46188.509431805556</v>
+        <v>46188.634431805556</v>
       </c>
       <c r="C27" s="9">
-        <v>46212.528463124996</v>
+        <v>46212.653463124996</v>
       </c>
       <c r="D27" s="9">
-        <v>46212.52846519676</v>
+        <v>46212.65346519676</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>108</v>
@@ -3125,13 +3125,13 @@
         <v>111</v>
       </c>
       <c r="B28" s="5">
-        <v>46188.50943740741</v>
+        <v>46188.63443740741</v>
       </c>
       <c r="C28" s="5">
-        <v>46212.528502280096</v>
+        <v>46212.653502280096</v>
       </c>
       <c r="D28" s="5">
-        <v>46212.52850395833</v>
+        <v>46212.65350395833</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>112</v>
@@ -3186,13 +3186,13 @@
         <v>114</v>
       </c>
       <c r="B29" s="9">
-        <v>46188.50951584491</v>
+        <v>46188.63451584491</v>
       </c>
       <c r="C29" s="9">
-        <v>46209.69373614583</v>
+        <v>46209.81873614583</v>
       </c>
       <c r="D29" s="9">
-        <v>46226.06869722222</v>
+        <v>46226.19369722222</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>115</v>
@@ -3251,13 +3251,13 @@
         <v>119</v>
       </c>
       <c r="B30" s="5">
-        <v>46188.50952219908</v>
+        <v>46188.63452219908</v>
       </c>
       <c r="C30" s="5">
-        <v>46209.693676319446</v>
+        <v>46209.818676319446</v>
       </c>
       <c r="D30" s="5">
-        <v>46209.69367788194</v>
+        <v>46209.81867788194</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>120</v>
@@ -3312,13 +3312,13 @@
         <v>122</v>
       </c>
       <c r="B31" s="9">
-        <v>46188.509528194445</v>
+        <v>46188.634528194445</v>
       </c>
       <c r="C31" s="9">
-        <v>46209.693722615746</v>
+        <v>46209.818722615746</v>
       </c>
       <c r="D31" s="9">
-        <v>46209.6937240625</v>
+        <v>46209.8187240625</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>123</v>
@@ -3373,13 +3373,13 @@
         <v>125</v>
       </c>
       <c r="B32" s="5">
-        <v>46188.50953408565</v>
+        <v>46188.63453408565</v>
       </c>
       <c r="C32" s="5">
-        <v>46209.694314988425</v>
+        <v>46209.819314988425</v>
       </c>
       <c r="D32" s="5">
-        <v>46226.06869837963</v>
+        <v>46226.19369837963</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>126</v>
@@ -3438,13 +3438,13 @@
         <v>128</v>
       </c>
       <c r="B33" s="9">
-        <v>46188.509538252314</v>
+        <v>46188.634538252314</v>
       </c>
       <c r="C33" s="9">
-        <v>46209.694259537035</v>
+        <v>46209.819259537035</v>
       </c>
       <c r="D33" s="9">
-        <v>46209.69426089121</v>
+        <v>46209.81926089121</v>
       </c>
       <c r="E33" s="10" t="s">
         <v>82</v>
@@ -3493,13 +3493,13 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46188.50954329861</v>
+        <v>46188.63454329861</v>
       </c>
       <c r="C34" s="5">
-        <v>46209.6943018287</v>
+        <v>46209.8193018287</v>
       </c>
       <c r="D34" s="5">
-        <v>46243.69722765047</v>
+        <v>46243.82222765047</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3548,13 +3548,13 @@
         <v>133</v>
       </c>
       <c r="B35" s="9">
-        <v>46188.50954804398</v>
+        <v>46188.63454804398</v>
       </c>
       <c r="C35" s="9">
-        <v>46209.49574709491</v>
+        <v>46209.62074709491</v>
       </c>
       <c r="D35" s="9">
-        <v>46254.07743388889</v>
+        <v>46254.20243388889</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>134</v>
@@ -3613,13 +3613,13 @@
         <v>138</v>
       </c>
       <c r="B36" s="5">
-        <v>46188.50955278936</v>
+        <v>46188.63455278936</v>
       </c>
       <c r="C36" s="5">
-        <v>46209.49502465277</v>
+        <v>46209.62002465277</v>
       </c>
       <c r="D36" s="5">
-        <v>46209.49502645833</v>
+        <v>46209.62002645833</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>88</v>
@@ -3668,13 +3668,13 @@
         <v>140</v>
       </c>
       <c r="B37" s="9">
-        <v>46188.50955811342</v>
+        <v>46188.63455811342</v>
       </c>
       <c r="C37" s="9">
-        <v>46209.49570212963</v>
+        <v>46209.62070212963</v>
       </c>
       <c r="D37" s="9">
-        <v>46209.495703761575</v>
+        <v>46209.620703761575</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>141</v>
@@ -3723,13 +3723,13 @@
         <v>143</v>
       </c>
       <c r="B38" s="5">
-        <v>46188.50956381945</v>
+        <v>46188.63456381945</v>
       </c>
       <c r="C38" s="5">
-        <v>46225.42480681713</v>
+        <v>46225.54980681713</v>
       </c>
       <c r="D38" s="5">
-        <v>46225.42480878472</v>
+        <v>46225.54980878472</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>144</v>
@@ -3778,13 +3778,13 @@
         <v>147</v>
       </c>
       <c r="B39" s="9">
-        <v>46188.50956738426</v>
+        <v>46188.63456738426</v>
       </c>
       <c r="C39" s="9">
-        <v>46209.69475005787</v>
+        <v>46209.81975005787</v>
       </c>
       <c r="D39" s="9">
-        <v>46226.06869717593</v>
+        <v>46226.19369717593</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>148</v>
@@ -3843,13 +3843,13 @@
         <v>150</v>
       </c>
       <c r="B40" s="5">
-        <v>46188.50957166667</v>
+        <v>46188.63457166667</v>
       </c>
       <c r="C40" s="5">
-        <v>46209.6946269676</v>
+        <v>46209.8196269676</v>
       </c>
       <c r="D40" s="5">
-        <v>46209.69462844907</v>
+        <v>46209.81962844907</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>85</v>
@@ -3898,13 +3898,13 @@
         <v>152</v>
       </c>
       <c r="B41" s="9">
-        <v>46188.509576701385</v>
+        <v>46188.634576701385</v>
       </c>
       <c r="C41" s="9">
-        <v>46209.694662615744</v>
+        <v>46209.819662615744</v>
       </c>
       <c r="D41" s="9">
-        <v>46209.69466414352</v>
+        <v>46209.81966414352</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>153</v>
@@ -3953,13 +3953,13 @@
         <v>155</v>
       </c>
       <c r="B42" s="5">
-        <v>46188.50917921297</v>
+        <v>46188.63417921297</v>
       </c>
       <c r="C42" s="5">
-        <v>46210.40449314815</v>
+        <v>46210.52949314815</v>
       </c>
       <c r="D42" s="5">
-        <v>46258.0634375</v>
+        <v>46258.1884375</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>156</v>
@@ -4006,13 +4006,13 @@
         <v>158</v>
       </c>
       <c r="B43" s="9">
-        <v>46188.50958247685</v>
+        <v>46188.63458247685</v>
       </c>
       <c r="C43" s="9">
-        <v>46196.39981820602</v>
+        <v>46196.52481820602</v>
       </c>
       <c r="D43" s="9">
-        <v>46258.038839733796</v>
+        <v>46258.163839733796</v>
       </c>
       <c r="E43" s="10" t="s">
         <v>159</v>
@@ -4071,13 +4071,13 @@
         <v>163</v>
       </c>
       <c r="B44" s="5">
-        <v>46188.509588587964</v>
+        <v>46188.634588587964</v>
       </c>
       <c r="C44" s="5">
-        <v>46198.38289115741</v>
+        <v>46198.50789115741</v>
       </c>
       <c r="D44" s="5">
-        <v>46258.038823379626</v>
+        <v>46258.163823379626</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>164</v>
@@ -4136,13 +4136,13 @@
         <v>166</v>
       </c>
       <c r="B45" s="9">
-        <v>46188.50959497685</v>
+        <v>46188.63459497685</v>
       </c>
       <c r="C45" s="9">
-        <v>46198.38295378472</v>
+        <v>46198.50795378472</v>
       </c>
       <c r="D45" s="9">
-        <v>46211.04538164352</v>
+        <v>46211.17038164352</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>78</v>
@@ -4201,13 +4201,13 @@
         <v>170</v>
       </c>
       <c r="B46" s="5">
-        <v>46188.50960983796</v>
+        <v>46188.63460983796</v>
       </c>
       <c r="C46" s="5">
-        <v>46258.41359034722</v>
+        <v>46258.53859034722</v>
       </c>
       <c r="D46" s="5">
-        <v>46260.06003548611</v>
+        <v>46260.18503548611</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>171</v>
@@ -4266,13 +4266,13 @@
         <v>176</v>
       </c>
       <c r="B47" s="9">
-        <v>46188.509613946764</v>
+        <v>46188.634613946764</v>
       </c>
       <c r="C47" s="9">
-        <v>46258.45212081019</v>
+        <v>46258.57712081019</v>
       </c>
       <c r="D47" s="9">
-        <v>46258.452122372684</v>
+        <v>46258.577122372684</v>
       </c>
       <c r="E47" s="10" t="s">
         <v>177</v>
@@ -4321,13 +4321,13 @@
         <v>180</v>
       </c>
       <c r="B48" s="5">
-        <v>46188.50961840278</v>
+        <v>46188.63461840278</v>
       </c>
       <c r="C48" s="5">
-        <v>46258.45213456018</v>
+        <v>46258.57713456018</v>
       </c>
       <c r="D48" s="5">
-        <v>46258.45213605324</v>
+        <v>46258.57713605324</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>177</v>
@@ -4376,13 +4376,13 @@
         <v>181</v>
       </c>
       <c r="B49" s="9">
-        <v>46188.50967295139</v>
+        <v>46188.63467295139</v>
       </c>
       <c r="C49" s="9">
-        <v>46258.44999196759</v>
+        <v>46258.57499196759</v>
       </c>
       <c r="D49" s="9">
-        <v>46258.45000517361</v>
+        <v>46258.57500517361</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>182</v>
@@ -4429,13 +4429,13 @@
         <v>184</v>
       </c>
       <c r="B50" s="5">
-        <v>46188.50967763889</v>
+        <v>46188.63467763889</v>
       </c>
       <c r="C50" s="5">
-        <v>46258.44988173612</v>
+        <v>46258.57488173612</v>
       </c>
       <c r="D50" s="5">
-        <v>46258.44990248843</v>
+        <v>46258.57490248843</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>185</v>
@@ -4494,13 +4494,13 @@
         <v>189</v>
       </c>
       <c r="B51" s="9">
-        <v>46188.509684942124</v>
+        <v>46188.634684942124</v>
       </c>
       <c r="C51" s="9">
-        <v>46258.44991376158</v>
+        <v>46258.57491376158</v>
       </c>
       <c r="D51" s="9">
-        <v>46258.44993045139</v>
+        <v>46258.57493045139</v>
       </c>
       <c r="E51" s="10" t="s">
         <v>190</v>
@@ -4559,13 +4559,13 @@
         <v>193</v>
       </c>
       <c r="B52" s="5">
-        <v>46188.509692962965</v>
+        <v>46188.634692962965</v>
       </c>
       <c r="C52" s="5">
-        <v>46258.44989256945</v>
+        <v>46258.57489256945</v>
       </c>
       <c r="D52" s="5">
-        <v>46258.44991056713</v>
+        <v>46258.57491056713</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>194</v>
@@ -4624,13 +4624,13 @@
         <v>196</v>
       </c>
       <c r="B53" s="9">
-        <v>46188.50969954861</v>
+        <v>46188.63469954861</v>
       </c>
       <c r="C53" s="9">
-        <v>46258.44995891204</v>
+        <v>46258.57495891204</v>
       </c>
       <c r="D53" s="9">
-        <v>46258.44997778935</v>
+        <v>46258.57497778935</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>197</v>
@@ -4689,13 +4689,13 @@
         <v>198</v>
       </c>
       <c r="B54" s="5">
-        <v>46188.50970560186</v>
+        <v>46188.63470560186</v>
       </c>
       <c r="C54" s="5">
-        <v>46258.44989766204</v>
+        <v>46258.57489766204</v>
       </c>
       <c r="D54" s="5">
-        <v>46258.44991270833</v>
+        <v>46258.57491270833</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4754,13 +4754,13 @@
         <v>201</v>
       </c>
       <c r="B55" s="9">
-        <v>46188.50971155093</v>
+        <v>46188.63471155093</v>
       </c>
       <c r="C55" s="9">
-        <v>46258.44997616898</v>
+        <v>46258.57497616898</v>
       </c>
       <c r="D55" s="9">
-        <v>46258.449992256945</v>
+        <v>46258.574992256945</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>200</v>
@@ -4819,13 +4819,13 @@
         <v>202</v>
       </c>
       <c r="B56" s="5">
-        <v>46188.50971731481</v>
+        <v>46188.63471731481</v>
       </c>
       <c r="C56" s="5">
-        <v>46258.45101996528</v>
+        <v>46258.57601996528</v>
       </c>
       <c r="D56" s="5">
-        <v>46258.45103575231</v>
+        <v>46258.57603575231</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>203</v>
@@ -4872,13 +4872,13 @@
         <v>205</v>
       </c>
       <c r="B57" s="9">
-        <v>46188.50972107639</v>
+        <v>46188.63472107639</v>
       </c>
       <c r="C57" s="9">
-        <v>46258.45006138889</v>
+        <v>46258.57506138889</v>
       </c>
       <c r="D57" s="9">
-        <v>46258.4500800463</v>
+        <v>46258.5750800463</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>206</v>
@@ -4937,13 +4937,13 @@
         <v>209</v>
       </c>
       <c r="B58" s="5">
-        <v>46188.50973258102</v>
+        <v>46188.63473258102</v>
       </c>
       <c r="C58" s="5">
-        <v>46258.4500391551</v>
+        <v>46258.5750391551</v>
       </c>
       <c r="D58" s="5">
-        <v>46258.45004092593</v>
+        <v>46258.57504092593</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>177</v>
@@ -4992,13 +4992,13 @@
         <v>212</v>
       </c>
       <c r="B59" s="9">
-        <v>46188.50974121528</v>
+        <v>46188.63474121528</v>
       </c>
       <c r="C59" s="9">
-        <v>46258.45004487269</v>
+        <v>46258.57504487269</v>
       </c>
       <c r="D59" s="9">
-        <v>46258.45004671296</v>
+        <v>46258.57504671296</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>177</v>
@@ -5047,13 +5047,13 @@
         <v>215</v>
       </c>
       <c r="B60" s="5">
-        <v>46188.50977284722</v>
+        <v>46188.63477284722</v>
       </c>
       <c r="C60" s="5">
-        <v>46258.450111886574</v>
+        <v>46258.575111886574</v>
       </c>
       <c r="D60" s="5">
-        <v>46258.45012483797</v>
+        <v>46258.57512483797</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>216</v>
@@ -5112,13 +5112,13 @@
         <v>217</v>
       </c>
       <c r="B61" s="9">
-        <v>46188.50977877315</v>
+        <v>46188.63477877315</v>
       </c>
       <c r="C61" s="9">
-        <v>46258.450087881945</v>
+        <v>46258.575087881945</v>
       </c>
       <c r="D61" s="9">
-        <v>46258.450089502316</v>
+        <v>46258.575089502316</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>177</v>
@@ -5167,13 +5167,13 @@
         <v>220</v>
       </c>
       <c r="B62" s="5">
-        <v>46188.50978605324</v>
+        <v>46188.63478605324</v>
       </c>
       <c r="C62" s="5">
-        <v>46258.4500969213</v>
+        <v>46258.5750969213</v>
       </c>
       <c r="D62" s="5">
-        <v>46258.45009857639</v>
+        <v>46258.57509857639</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>177</v>
@@ -5222,13 +5222,13 @@
         <v>221</v>
       </c>
       <c r="B63" s="9">
-        <v>46188.50985537037</v>
+        <v>46188.63485537037</v>
       </c>
       <c r="C63" s="9">
-        <v>46258.450180775464</v>
+        <v>46258.575180775464</v>
       </c>
       <c r="D63" s="9">
-        <v>46258.45019108796</v>
+        <v>46258.57519108796</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>222</v>
@@ -5287,13 +5287,13 @@
         <v>223</v>
       </c>
       <c r="B64" s="5">
-        <v>46188.509861805556</v>
+        <v>46188.634861805556</v>
       </c>
       <c r="C64" s="5">
-        <v>46258.45013146991</v>
+        <v>46258.57513146991</v>
       </c>
       <c r="D64" s="5">
-        <v>46258.45013333333</v>
+        <v>46258.57513333333</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>177</v>
@@ -5342,13 +5342,13 @@
         <v>225</v>
       </c>
       <c r="B65" s="9">
-        <v>46188.50986881944</v>
+        <v>46188.63486881944</v>
       </c>
       <c r="C65" s="9">
-        <v>46258.450166423616</v>
+        <v>46258.575166423616</v>
       </c>
       <c r="D65" s="9">
-        <v>46258.45016814815</v>
+        <v>46258.57516814815</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>177</v>
@@ -5397,13 +5397,13 @@
         <v>226</v>
       </c>
       <c r="B66" s="5">
-        <v>46188.50989331018</v>
+        <v>46188.63489331018</v>
       </c>
       <c r="C66" s="5">
-        <v>46258.45025863426</v>
+        <v>46258.57525863426</v>
       </c>
       <c r="D66" s="5">
-        <v>46265.2187968287</v>
+        <v>46265.3437968287</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>182</v>
@@ -5450,13 +5450,13 @@
         <v>228</v>
       </c>
       <c r="B67" s="9">
-        <v>46188.509903391205</v>
+        <v>46188.634903391205</v>
       </c>
       <c r="C67" s="9">
-        <v>46212.52878395833</v>
+        <v>46212.65378395833</v>
       </c>
       <c r="D67" s="9">
-        <v>46212.52919707176</v>
+        <v>46212.65419707176</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>229</v>
@@ -5515,13 +5515,13 @@
         <v>230</v>
       </c>
       <c r="B68" s="5">
-        <v>46188.5099100463</v>
+        <v>46188.6349100463</v>
       </c>
       <c r="C68" s="5">
-        <v>46212.529018402776</v>
+        <v>46212.654018402776</v>
       </c>
       <c r="D68" s="5">
-        <v>46212.52911137731</v>
+        <v>46212.65411137731</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>231</v>
@@ -5580,13 +5580,13 @@
         <v>232</v>
       </c>
       <c r="B69" s="9">
-        <v>46188.5099165162</v>
+        <v>46188.6349165162</v>
       </c>
       <c r="C69" s="9">
-        <v>46258.45024318287</v>
+        <v>46258.57524318287</v>
       </c>
       <c r="D69" s="9">
-        <v>46258.450258171295</v>
+        <v>46258.575258171295</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>233</v>
@@ -5645,13 +5645,13 @@
         <v>234</v>
       </c>
       <c r="B70" s="5">
-        <v>46188.509922916666</v>
+        <v>46188.634922916666</v>
       </c>
       <c r="C70" s="5">
-        <v>46225.424930995374</v>
+        <v>46225.549930995374</v>
       </c>
       <c r="D70" s="5">
-        <v>46255.08034878472</v>
+        <v>46255.20534878472</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>235</v>
@@ -5710,11 +5710,11 @@
         <v>237</v>
       </c>
       <c r="B71" s="9">
-        <v>46188.50992795139</v>
+        <v>46188.63492795139</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="9">
-        <v>46258.45097358796</v>
+        <v>46258.57597358796</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>238</v>
@@ -5757,13 +5757,13 @@
         <v>240</v>
       </c>
       <c r="B72" s="5">
-        <v>46188.50993152778</v>
+        <v>46188.63493152778</v>
       </c>
       <c r="C72" s="5">
-        <v>46258.450706250005</v>
+        <v>46258.575706250005</v>
       </c>
       <c r="D72" s="5">
-        <v>46258.45072197917</v>
+        <v>46258.57572197917</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>241</v>
@@ -5822,11 +5822,11 @@
         <v>243</v>
       </c>
       <c r="B73" s="9">
-        <v>46188.50994034723</v>
+        <v>46188.63494034723</v>
       </c>
       <c r="C73" s="10"/>
       <c r="D73" s="9">
-        <v>46258.45014153935</v>
+        <v>46258.57514153935</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>177</v>
@@ -5875,11 +5875,11 @@
         <v>245</v>
       </c>
       <c r="B74" s="5">
-        <v>46188.509945150465</v>
+        <v>46188.634945150465</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46258.45017729167</v>
+        <v>46258.57517729167</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>177</v>
@@ -5928,13 +5928,13 @@
         <v>246</v>
       </c>
       <c r="B75" s="9">
-        <v>46188.509963668985</v>
+        <v>46188.634963668985</v>
       </c>
       <c r="C75" s="9">
-        <v>46197.46204829861</v>
+        <v>46197.58704829861</v>
       </c>
       <c r="D75" s="9">
-        <v>46258.03920450232</v>
+        <v>46258.16420450232</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>247</v>
@@ -5993,13 +5993,13 @@
         <v>248</v>
       </c>
       <c r="B76" s="5">
-        <v>46188.50996887732</v>
+        <v>46188.63496887732</v>
       </c>
       <c r="C76" s="5">
-        <v>46197.46195519676</v>
+        <v>46197.58695519676</v>
       </c>
       <c r="D76" s="5">
-        <v>46223.43883306713</v>
+        <v>46223.56383306713</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>177</v>
@@ -6048,13 +6048,13 @@
         <v>251</v>
       </c>
       <c r="B77" s="9">
-        <v>46188.50998112268</v>
+        <v>46188.63498112268</v>
       </c>
       <c r="C77" s="9">
-        <v>46197.462035335644</v>
+        <v>46197.587035335644</v>
       </c>
       <c r="D77" s="9">
-        <v>46223.438828865736</v>
+        <v>46223.563828865736</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>177</v>
@@ -6103,13 +6103,13 @@
         <v>253</v>
       </c>
       <c r="B78" s="5">
-        <v>46188.510046296295</v>
+        <v>46188.635046296295</v>
       </c>
       <c r="C78" s="5">
-        <v>46258.45088525463</v>
+        <v>46258.57588525463</v>
       </c>
       <c r="D78" s="5">
-        <v>46258.45089622685</v>
+        <v>46258.57589622685</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>254</v>
@@ -6168,13 +6168,13 @@
         <v>255</v>
       </c>
       <c r="B79" s="9">
-        <v>46188.51005403935</v>
+        <v>46188.63505403935</v>
       </c>
       <c r="C79" s="9">
-        <v>46258.45086165509</v>
+        <v>46258.57586165509</v>
       </c>
       <c r="D79" s="9">
-        <v>46258.45086484954</v>
+        <v>46258.57586484954</v>
       </c>
       <c r="E79" s="10" t="s">
         <v>177</v>
@@ -6223,13 +6223,13 @@
         <v>257</v>
       </c>
       <c r="B80" s="5">
-        <v>46188.51006813657</v>
+        <v>46188.63506813657</v>
       </c>
       <c r="C80" s="5">
-        <v>46258.45087064814</v>
+        <v>46258.57587064814</v>
       </c>
       <c r="D80" s="5">
-        <v>46258.45087212963</v>
+        <v>46258.57587212963</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>177</v>
@@ -6278,13 +6278,13 @@
         <v>259</v>
       </c>
       <c r="B81" s="9">
-        <v>46188.51009704861</v>
+        <v>46188.63509704861</v>
       </c>
       <c r="C81" s="9">
-        <v>46258.45092091435</v>
+        <v>46258.57592091435</v>
       </c>
       <c r="D81" s="9">
-        <v>46258.45093314815</v>
+        <v>46258.57593314815</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>260</v>
@@ -6343,13 +6343,13 @@
         <v>261</v>
       </c>
       <c r="B82" s="5">
-        <v>46188.510102939814</v>
+        <v>46188.635102939814</v>
       </c>
       <c r="C82" s="5">
-        <v>46258.45090001158</v>
+        <v>46258.57590001158</v>
       </c>
       <c r="D82" s="5">
-        <v>46258.450901539356</v>
+        <v>46258.575901539356</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>177</v>
@@ -6398,13 +6398,13 @@
         <v>264</v>
       </c>
       <c r="B83" s="9">
-        <v>46188.51010991898</v>
+        <v>46188.63510991898</v>
       </c>
       <c r="C83" s="9">
-        <v>46258.45090351852</v>
+        <v>46258.57590351852</v>
       </c>
       <c r="D83" s="9">
-        <v>46258.45090449074</v>
+        <v>46258.57590449074</v>
       </c>
       <c r="E83" s="10" t="s">
         <v>177</v>
@@ -6453,13 +6453,13 @@
         <v>266</v>
       </c>
       <c r="B84" s="5">
-        <v>46188.51013603009</v>
+        <v>46188.63513603009</v>
       </c>
       <c r="C84" s="5">
-        <v>46258.45096667824</v>
+        <v>46258.57596667824</v>
       </c>
       <c r="D84" s="5">
-        <v>46259.04779440972</v>
+        <v>46259.17279440972</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>267</v>
@@ -6518,13 +6518,13 @@
         <v>269</v>
       </c>
       <c r="B85" s="9">
-        <v>46188.51014172454</v>
+        <v>46188.63514172454</v>
       </c>
       <c r="C85" s="9">
-        <v>46258.450944502314</v>
+        <v>46258.575944502314</v>
       </c>
       <c r="D85" s="9">
-        <v>46258.45094594907</v>
+        <v>46258.57594594907</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>178</v>
@@ -6573,13 +6573,13 @@
         <v>271</v>
       </c>
       <c r="B86" s="5">
-        <v>46188.51014853009</v>
+        <v>46188.63514853009</v>
       </c>
       <c r="C86" s="5">
-        <v>46258.450951631945</v>
+        <v>46258.575951631945</v>
       </c>
       <c r="D86" s="5">
-        <v>46258.45095326389</v>
+        <v>46258.57595326389</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>177</v>
@@ -6628,11 +6628,11 @@
         <v>272</v>
       </c>
       <c r="B87" s="9">
-        <v>46188.51021115741</v>
+        <v>46188.63521115741</v>
       </c>
       <c r="C87" s="10"/>
       <c r="D87" s="9">
-        <v>46261.04323309028</v>
+        <v>46261.16823309028</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>273</v>
@@ -6691,11 +6691,11 @@
         <v>275</v>
       </c>
       <c r="B88" s="5">
-        <v>46188.51021795139</v>
+        <v>46188.63521795139</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46261.04292226852</v>
+        <v>46261.16792226852</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>177</v>
@@ -6744,11 +6744,11 @@
         <v>277</v>
       </c>
       <c r="B89" s="9">
-        <v>46188.510222916666</v>
+        <v>46188.635222916666</v>
       </c>
       <c r="C89" s="10"/>
       <c r="D89" s="9">
-        <v>46260.04338662037</v>
+        <v>46260.16838662037</v>
       </c>
       <c r="E89" s="10" t="s">
         <v>177</v>
@@ -6797,11 +6797,11 @@
         <v>278</v>
       </c>
       <c r="B90" s="5">
-        <v>46188.510247199076</v>
+        <v>46188.635247199076</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46260.464834479164</v>
+        <v>46260.589834479164</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>279</v>
@@ -6844,11 +6844,11 @@
         <v>281</v>
       </c>
       <c r="B91" s="9">
-        <v>46188.510250844905</v>
+        <v>46188.635250844905</v>
       </c>
       <c r="C91" s="10"/>
       <c r="D91" s="9">
-        <v>46262.061115115735</v>
+        <v>46262.186115115735</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>282</v>
@@ -6907,11 +6907,11 @@
         <v>286</v>
       </c>
       <c r="B92" s="5">
-        <v>46188.51025673611</v>
+        <v>46188.63525673611</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46261.042970636576</v>
+        <v>46261.167970636576</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>177</v>
@@ -6960,11 +6960,11 @@
         <v>288</v>
       </c>
       <c r="B93" s="9">
-        <v>46188.510261689815</v>
+        <v>46188.635261689815</v>
       </c>
       <c r="C93" s="10"/>
       <c r="D93" s="9">
-        <v>46261.04297177083</v>
+        <v>46261.16797177083</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>177</v>
@@ -7013,11 +7013,11 @@
         <v>289</v>
       </c>
       <c r="B94" s="5">
-        <v>46188.510279375</v>
+        <v>46188.635279375</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46263.07801833333</v>
+        <v>46263.20301833333</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>290</v>
@@ -7076,11 +7076,11 @@
         <v>291</v>
       </c>
       <c r="B95" s="9">
-        <v>46188.51028446759</v>
+        <v>46188.63528446759</v>
       </c>
       <c r="C95" s="10"/>
       <c r="D95" s="9">
-        <v>46262.044073287034</v>
+        <v>46262.169073287034</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>177</v>
@@ -7129,11 +7129,11 @@
         <v>293</v>
       </c>
       <c r="B96" s="5">
-        <v>46188.5102894213</v>
+        <v>46188.6352894213</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46262.04407469908</v>
+        <v>46262.16907469908</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>177</v>
@@ -7182,11 +7182,11 @@
         <v>295</v>
       </c>
       <c r="B97" s="9">
-        <v>46188.51030922454</v>
+        <v>46188.63530922454</v>
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="9">
-        <v>46266.064001018516</v>
+        <v>46266.189001018516</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>296</v>
@@ -7245,11 +7245,11 @@
         <v>297</v>
       </c>
       <c r="B98" s="5">
-        <v>46188.51031412037</v>
+        <v>46188.63531412037</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46265.04404490741</v>
+        <v>46265.16904490741</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>177</v>
@@ -7298,11 +7298,11 @@
         <v>299</v>
       </c>
       <c r="B99" s="9">
-        <v>46188.51032239583</v>
+        <v>46188.63532239583</v>
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="9">
-        <v>46265.0440515625</v>
+        <v>46265.1690515625</v>
       </c>
       <c r="E99" s="10" t="s">
         <v>177</v>
@@ -7351,11 +7351,11 @@
         <v>300</v>
       </c>
       <c r="B100" s="5">
-        <v>46188.51038068287</v>
+        <v>46188.63538068287</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46267.04507989583</v>
+        <v>46267.17007989583</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>301</v>
@@ -7414,11 +7414,11 @@
         <v>303</v>
       </c>
       <c r="B101" s="9">
-        <v>46188.5103874537</v>
+        <v>46188.6353874537</v>
       </c>
       <c r="C101" s="10"/>
       <c r="D101" s="9">
-        <v>46266.043580185185</v>
+        <v>46266.168580185185</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>177</v>
@@ -7467,11 +7467,11 @@
         <v>304</v>
       </c>
       <c r="B102" s="5">
-        <v>46188.51039206018</v>
+        <v>46188.63539206018</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46266.043581412036</v>
+        <v>46266.168581412036</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>177</v>
@@ -7520,11 +7520,11 @@
         <v>305</v>
       </c>
       <c r="B103" s="9">
-        <v>46188.510410682866</v>
+        <v>46188.635410682866</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="9">
-        <v>46188.54623894676</v>
+        <v>46188.67123894676</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>306</v>
@@ -7567,11 +7567,11 @@
         <v>308</v>
       </c>
       <c r="B104" s="5">
-        <v>46188.510413993055</v>
+        <v>46188.635413993055</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46276.00725435185</v>
+        <v>46276.13225435185</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>309</v>
@@ -7630,11 +7630,11 @@
         <v>312</v>
       </c>
       <c r="B105" s="9">
-        <v>46188.51041944444</v>
+        <v>46188.63541944444</v>
       </c>
       <c r="C105" s="10"/>
       <c r="D105" s="9">
-        <v>46276.007254571756</v>
+        <v>46276.132254571756</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>313</v>

</xml_diff>